<commit_message>
updated CPI MCP configuration and create batch execution agent
</commit_message>
<xml_diff>
--- a/backend/src/config/test.xlsx
+++ b/backend/src/config/test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saura\Downloads\AI Basics (Dev)\Utilities via Claude\LearnViaClaude\AgenticCPITool\AgenticCPITool\backend\src\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6D587B11-2D08-4B49-9AAC-D6C390A5B538}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E4D1BEC-88CD-4AA3-B9F4-E32984791360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C08536B2-4956-474F-98A1-2729EECC5616}"/>
   </bookViews>
@@ -48,25 +48,25 @@
     <t>Deploy</t>
   </si>
   <si>
-    <t>Demo</t>
-  </si>
-  <si>
-    <t>param0</t>
-  </si>
-  <si>
     <t>no</t>
   </si>
   <si>
     <t>Demo_CheckAdapters</t>
   </si>
   <si>
-    <t>param1</t>
-  </si>
-  <si>
     <t>yes</t>
   </si>
   <si>
-    <t>param2</t>
+    <t>prop1</t>
+  </si>
+  <si>
+    <t>prop2</t>
+  </si>
+  <si>
+    <t>prop0</t>
+  </si>
+  <si>
+    <t>demo</t>
   </si>
 </sst>
 </file>
@@ -441,38 +441,38 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
-        <v>8</v>
-      </c>
       <c r="C2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C3">
-        <v>2</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
         <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>